<commit_message>
finished Zeitstrahl mit Kriminellen Nachrichten
</commit_message>
<xml_diff>
--- a/Zeitstrahl.xlsx
+++ b/Zeitstrahl.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\amonb\OneDrive\Dokumente\Semester II\Der Sachverstädnige vor Gericht\Git Repository\sachverst-ndiger\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A6986B0E-525B-4D2C-8A87-7E9BBED25577}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D2E797F-078D-4376-A5BC-D5F7FB9CC032}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="15495" yWindow="-21600" windowWidth="19410" windowHeight="20985" xr2:uid="{F14C7C15-811B-4F1F-80F2-413CDD7532BB}"/>
+    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{F14C7C15-811B-4F1F-80F2-413CDD7532BB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="554" uniqueCount="257">
   <si>
     <t>15.02.2021</t>
   </si>
@@ -360,6 +360,453 @@
   </si>
   <si>
     <t>Check it out. That house was loaded. Easy access via the garage ≡ƒæî</t>
+  </si>
+  <si>
+    <t>06.03.2021</t>
+  </si>
+  <si>
+    <t>46702578150@s.whatsapp.net</t>
+  </si>
+  <si>
+    <t>You are slightly cute</t>
+  </si>
+  <si>
+    <t>1643401562</t>
+  </si>
+  <si>
+    <t>Ouch missy! Cruel but probably true. Missing you already...</t>
+  </si>
+  <si>
+    <t>Rupert Beae</t>
+  </si>
+  <si>
+    <t>100063691416962</t>
+  </si>
+  <si>
+    <t>U likey da bling baby?</t>
+  </si>
+  <si>
+    <t>Gooooosssse</t>
+  </si>
+  <si>
+    <t>351760022</t>
+  </si>
+  <si>
+    <t>07.03.2021</t>
+  </si>
+  <si>
+    <t>OK deal. Send the money ≡ƒÆ░ usual place, usual time.</t>
+  </si>
+  <si>
+    <t>Anyone want to play in the big league. Can you guys move this stuff if we come across some?</t>
+  </si>
+  <si>
+    <t>Twi Grey</t>
+  </si>
+  <si>
+    <t>Score!</t>
+  </si>
+  <si>
+    <t>So sweet , what a score. You hit the big time with that baby</t>
+  </si>
+  <si>
+    <t>Yep going back there soon. Know a guy who will take it off our hands after the job is done. Make some extra cash on top of the big loot.</t>
+  </si>
+  <si>
+    <t>08.03.2021</t>
+  </si>
+  <si>
+    <t>Location-sharing ended</t>
+  </si>
+  <si>
+    <t>Good security at this place ≡ƒæÅ</t>
+  </si>
+  <si>
+    <t>Twilight Grey</t>
+  </si>
+  <si>
+    <t>Give me the rings≡ƒÿì≡ƒÿì</t>
+  </si>
+  <si>
+    <t>How exciting! Do let me know when you are planning to be dangerous again. I would like to watch you at your finest...</t>
+  </si>
+  <si>
+    <t>09.03.2021</t>
+  </si>
+  <si>
+    <t>Awesome. Looks like a perfect target. Thanks Twilight you rock ≡ƒ¬¿≡ƒÄ╕</t>
+  </si>
+  <si>
+    <t>Twilight G</t>
+  </si>
+  <si>
+    <t>This place has easy access from.the woods behind it. Should be good cover for a job.</t>
+  </si>
+  <si>
+    <t>Nice ok let's make the plan. We need tools and shit...</t>
+  </si>
+  <si>
+    <t>10.03.2021</t>
+  </si>
+  <si>
+    <t>I got a few things to buy and sell. I can fence some of your gear if you like? What u got dude....</t>
+  </si>
+  <si>
+    <t>I need to see this stuff in person and check the quality of the merchandise. For all I know you just downloaded this shit off the internet. Not that I don't trust you but I don't....</t>
+  </si>
+  <si>
+    <t>Shame. OK well let me know if you ever want picking up and lifted to new heights ≡ƒÿà</t>
+  </si>
+  <si>
+    <t>Let's just say that last night out score was quantity over quality....</t>
+  </si>
+  <si>
+    <t>11.03.2021</t>
+  </si>
+  <si>
+    <t>Ok this is our secret stash location. We hide the loot here in future to avoid the risk of being caught in possession....</t>
+  </si>
+  <si>
+    <t>Maverick wants to sell gear to BigBoss</t>
+  </si>
+  <si>
+    <t>Stash location is cool</t>
+  </si>
+  <si>
+    <t>This place was very isolated</t>
+  </si>
+  <si>
+    <t>This one for a getaway vehicle?</t>
+  </si>
+  <si>
+    <t>Yes but naturally keep it quiet. Don't want the whole world to know about this place...</t>
+  </si>
+  <si>
+    <t>12.03.2021</t>
+  </si>
+  <si>
+    <t>IΓÇÖm meeting a contact later...any bling to move</t>
+  </si>
+  <si>
+    <t>Big Boss</t>
+  </si>
+  <si>
+    <t>Meet me at the rocket ship tonight...</t>
+  </si>
+  <si>
+    <t>Maverick.4444</t>
+  </si>
+  <si>
+    <t>u44afa6f6317115c622a22eaac029f7f9</t>
+  </si>
+  <si>
+    <t>Dude stop being a moron. Grab the stolen goods and get back to base.</t>
+  </si>
+  <si>
+    <t>13.03.2021</t>
+  </si>
+  <si>
+    <t>It was a good week. We pay off our debts soon boss ≡ƒÿÄ</t>
+  </si>
+  <si>
+    <t>Celebrate with a pair of diamond earrings?</t>
+  </si>
+  <si>
+    <t>14.03.2021</t>
+  </si>
+  <si>
+    <t>Michael Jonson</t>
+  </si>
+  <si>
+    <t>This could be a good place to visit ...</t>
+  </si>
+  <si>
+    <t>Scored!!!</t>
+  </si>
+  <si>
+    <t>Another jackpot house today. It's too easy....</t>
+  </si>
+  <si>
+    <t>It used to be a bank but I recon they still hold some really valuable things there</t>
+  </si>
+  <si>
+    <t>15.03.2021</t>
+  </si>
+  <si>
+    <t>That's what you get for wearing pink pants</t>
+  </si>
+  <si>
+    <t>16.03.2021</t>
+  </si>
+  <si>
+    <t>Hey dudes. This sucks. Big boss is giving us less and less for each score. Told me  price of gold is going down....</t>
+  </si>
+  <si>
+    <t>We may have to switch jobs...</t>
+  </si>
+  <si>
+    <t>I want to trade. The boys let me know you deal in cheap gear and occasionally I get some to sell and every now and then I need to buy...</t>
+  </si>
+  <si>
+    <t>OK but how can I trust you after last time? You really screwed up...</t>
+  </si>
+  <si>
+    <t>Seriously you can trust me. I won't make the same mistake twice. I will pay on time and keep your secrets. In my honor</t>
+  </si>
+  <si>
+    <t>That scumbag Bad Boy is back. Wants to play nice and join the gang? What do u think? ≡ƒÿ│</t>
+  </si>
+  <si>
+    <t>Ah man. Really? He has a bad rep.\nDropped people right in it before. You know the rumours... I dunno man.</t>
+  </si>
+  <si>
+    <t>Ah shit. Yer I guess so. Tooled up already? Man it's like you knew already? ≡ƒÿÅ</t>
+  </si>
+  <si>
+    <t>17.03.2021</t>
+  </si>
+  <si>
+    <t>Going soon.... hoping to bring the real deal</t>
+  </si>
+  <si>
+    <t>OK Bad Boy... Goose agreed to give you a second chance,  but you need to do everything we say OK?</t>
+  </si>
+  <si>
+    <t>First job. Find us a place to rob..</t>
+  </si>
+  <si>
+    <t>Ok boss will do...</t>
+  </si>
+  <si>
+    <t>Heard something from Twilight and got nervous</t>
+  </si>
+  <si>
+    <t>This is a nice piece I got. What do you guys think?</t>
+  </si>
+  <si>
+    <t>18.03.2021</t>
+  </si>
+  <si>
+    <t>50% Still owed. You forget about the interest outstanding...</t>
+  </si>
+  <si>
+    <t>19.03.2021</t>
+  </si>
+  <si>
+    <t>Goose.4444</t>
+  </si>
+  <si>
+    <t>Good getaway thingy in the city</t>
+  </si>
+  <si>
+    <t>So what's it going to take to get a clean break ?</t>
+  </si>
+  <si>
+    <t>BigBoss</t>
+  </si>
+  <si>
+    <t>Nice work Mav. What is the cut?</t>
+  </si>
+  <si>
+    <t>This little bag of white powder could be worth 100,000kr if we deal with it correctly ≡ƒñö</t>
+  </si>
+  <si>
+    <t>20.03.2021</t>
+  </si>
+  <si>
+    <t>He even does rocks now?</t>
+  </si>
+  <si>
+    <t>What happens if I say the word heroin in this chat thread ≡ƒº╡???</t>
+  </si>
+  <si>
+    <t>Maybe try selling crack instead?</t>
+  </si>
+  <si>
+    <t>Funnily enough I have a kilo of white powder available...</t>
+  </si>
+  <si>
+    <t>Well how convenient?\nSo what's the price of that then?</t>
+  </si>
+  <si>
+    <t>OK boss I have a possible big score coming in via a contact. Could be worth 100,000 to clear my debts!!!</t>
+  </si>
+  <si>
+    <t>You don't want me to have to send the big boys around again to your place, do you?</t>
+  </si>
+  <si>
+    <t>Yes well finest quality,  very cheap to you my friend. You can cut it down and quadruple the value...</t>
+  </si>
+  <si>
+    <t>21.03.2021</t>
+  </si>
+  <si>
+    <t>OK okay. I get the message. I will pay. Need 48hrs. Got a big deal for white powder in the works.</t>
+  </si>
+  <si>
+    <t>23.03.2021</t>
+  </si>
+  <si>
+    <t>3k with necklace</t>
+  </si>
+  <si>
+    <t>This one looks like a great target. Close to the woods for an easy getaway in multiple directions ≡ƒÿî≡ƒæî</t>
+  </si>
+  <si>
+    <t>OK we will hit this one again  tonight. It was an easy target last time and the gap is large enough for the insurance payout to replace the stuff we stole first time around....</t>
+  </si>
+  <si>
+    <t>Give me 5 mins to grab tools</t>
+  </si>
+  <si>
+    <t>Last night was a good hit</t>
+  </si>
+  <si>
+    <t>24.03.2021</t>
+  </si>
+  <si>
+    <t>I will be there bring the cash and you get the delivery of powder....</t>
+  </si>
+  <si>
+    <t>So is the deal going down tonight?</t>
+  </si>
+  <si>
+    <t>Yes boss. I'm on route to make the deal now.</t>
+  </si>
+  <si>
+    <t>If it goes to shit, this is where I am\n..</t>
+  </si>
+  <si>
+    <t>OK I'm here now. Black jacket. Where are you at???</t>
+  </si>
+  <si>
+    <t>Damn! I need a truck this bag to carry all the money we just made !!!!</t>
+  </si>
+  <si>
+    <t>25.03.2021</t>
+  </si>
+  <si>
+    <t>Time to celebrate gang,. MR BIG is paid off finally ≡ƒÖî</t>
+  </si>
+  <si>
+    <t>Be there and fast. I won't wait any longer for my money. Don't make me come and take it by force...</t>
+  </si>
+  <si>
+    <t>Ok heading out with Mav on another round of robbing the neighborhood ≡ƒÿè</t>
+  </si>
+  <si>
+    <t>26.03.2021</t>
+  </si>
+  <si>
+    <t>Make it a week. This stuff is selling so fast I can't keep up. Need new packages asap</t>
+  </si>
+  <si>
+    <t>27.03.2021</t>
+  </si>
+  <si>
+    <t>Oh no run</t>
+  </si>
+  <si>
+    <t>When can you get me more white powder?</t>
+  </si>
+  <si>
+    <t>Hmmm, my contact wasnΓÇÖt here today</t>
+  </si>
+  <si>
+    <t>I need more white lines, this big!</t>
+  </si>
+  <si>
+    <t>Oh yes.... we hit the jackpot tonight team ≡ƒñ¬</t>
+  </si>
+  <si>
+    <t>They had gold blocks in the house! Unreal....</t>
+  </si>
+  <si>
+    <t>28.03.2021</t>
+  </si>
+  <si>
+    <t>Hey you looking for a safe cracker?</t>
+  </si>
+  <si>
+    <t>29.03.2021</t>
+  </si>
+  <si>
+    <t>You still in the market ???</t>
+  </si>
+  <si>
+    <t>Not as big a quantity available this time. 15,000kr for 100 grams</t>
+  </si>
+  <si>
+    <t>Yes deal. I get cash in 24hrs . Can we meet tomorrow at location you choose???</t>
+  </si>
+  <si>
+    <t>Good place to stash the next stolen car... ≡ƒÿÅ</t>
+  </si>
+  <si>
+    <t>This place is perfect.  Backs.onto the woods for an easy escape.. nothing overlooked</t>
+  </si>
+  <si>
+    <t>Ok cool. Last one for the evening. My stash bag is already full ≡ƒÿî</t>
+  </si>
+  <si>
+    <t>Yes obviously.  15,000kr is the deal. I will be there.</t>
+  </si>
+  <si>
+    <t>30.03.2021</t>
+  </si>
+  <si>
+    <t>OK gang. Going to make second drop with Bad Boy for the coke. Have my back I will go there with the package. Goose cover my back dude...</t>
+  </si>
+  <si>
+    <t>31.03.2021</t>
+  </si>
+  <si>
+    <t>Want to make some more money? I have a job for you, if you're interested...</t>
+  </si>
+  <si>
+    <t>1224624669</t>
+  </si>
+  <si>
+    <t>Do you want me to fence some gear?</t>
+  </si>
+  <si>
+    <t>More white.lines</t>
+  </si>
+  <si>
+    <t>Fuck you Goose. This is between me and you. Don't bring the others into it.</t>
+  </si>
+  <si>
+    <t>Oh god Goldy. Please stop using the product. We can't afford it and I don't know if I can rely on you. Need your head straight while Goose is wobbling....</t>
+  </si>
+  <si>
+    <t>01.04.2021</t>
+  </si>
+  <si>
+    <t>Hey all. Goose isn't talking to me, but there's still work to be done. I am going out for a recon. Looking for business as usual...</t>
+  </si>
+  <si>
+    <t>Hey. If you hear from Goose, let me know please.  We had a disagreement.  Want to make sure he doesn't start doing deals behind my back.... I am your supplier OK???</t>
+  </si>
+  <si>
+    <t>No man. Didn't notice the date until now. This is straight up serious. We have internal issues. No problem for you, but only talk to me OK???</t>
+  </si>
+  <si>
+    <t>Hey man can you come to Stockholm. I got 2 jobs for you. Soon as you like. I will pay premium rates.</t>
+  </si>
+  <si>
+    <t>Got some trouble with a dealer and a former partner.  Need them both taken care of.</t>
+  </si>
+  <si>
+    <t>Mike Jonson</t>
+  </si>
+  <si>
+    <t>Dude are you crazy?\n1. Never discuss that type of business in chat\n2. There is a global pandemic on, bit hard to travel at short notice.\nThis is something you need to fix yourself locally.\nNo can do.</t>
+  </si>
+  <si>
+    <t>02.04.2021</t>
+  </si>
+  <si>
+    <t>Boss I have cops outside the house. Help me please. Think Goose has ratted us out.....</t>
   </si>
 </sst>
 </file>
@@ -436,12 +883,12 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="22" fontId="0" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -776,7 +1223,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{419F6C20-9CB3-4D32-915F-78A5F233F1E4}">
-  <dimension ref="A1:K100"/>
+  <dimension ref="A1:U267"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
@@ -976,7 +1423,7 @@
       </c>
     </row>
     <row r="48" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A48" s="2" t="s">
+      <c r="A48" t="s">
         <v>40</v>
       </c>
       <c r="K48" t="s">
@@ -984,7 +1431,7 @@
       </c>
     </row>
     <row r="49" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A49" s="2" t="s">
+      <c r="A49" t="s">
         <v>41</v>
       </c>
       <c r="K49" t="s">
@@ -992,7 +1439,7 @@
       </c>
     </row>
     <row r="50" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A50" s="2" t="s">
+      <c r="A50" t="s">
         <v>42</v>
       </c>
       <c r="K50" t="s">
@@ -1000,17 +1447,17 @@
       </c>
     </row>
     <row r="51" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A51" s="2" t="s">
+      <c r="A51" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="52" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A52" s="2" t="s">
+      <c r="A52" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="53" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A53" s="2" t="s">
+      <c r="A53" t="s">
         <v>50</v>
       </c>
       <c r="H53" t="s">
@@ -1018,7 +1465,7 @@
       </c>
     </row>
     <row r="54" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A54" s="2" t="s">
+      <c r="A54" t="s">
         <v>52</v>
       </c>
     </row>
@@ -1155,247 +1602,1763 @@
         <v>80</v>
       </c>
     </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A81" s="3" t="s">
+    <row r="81" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A81" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="B81" s="4" t="s">
+      <c r="B81" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="C81" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="D81" s="4" t="s">
+      <c r="C81" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="D81" s="3" t="s">
         <v>83</v>
       </c>
-      <c r="E81" s="4" t="s">
+      <c r="E81" s="3" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A82" s="5" t="s">
+    <row r="82" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A82" s="4" t="s">
         <v>81</v>
       </c>
-      <c r="B82" s="6" t="s">
+      <c r="B82" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="C82" s="6" t="s">
-        <v>59</v>
-      </c>
-      <c r="D82" s="6" t="s">
+      <c r="C82" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="D82" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="E82" s="6" t="s">
+      <c r="E82" s="5" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A83" s="5" t="s">
+    <row r="83" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A83" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="B83" s="6" t="s">
+      <c r="B83" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="C83" s="6" t="s">
-        <v>59</v>
-      </c>
-      <c r="D83" s="6" t="s">
+      <c r="C83" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="D83" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="E83" s="6" t="s">
+      <c r="E83" s="5" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A84" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="B84" s="6" t="s">
+    <row r="84" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A84" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B84" s="5" t="s">
         <v>91</v>
       </c>
-      <c r="C84" s="6" t="s">
+      <c r="C84" s="5" t="s">
         <v>94</v>
       </c>
-      <c r="D84" s="6" t="s">
+      <c r="D84" s="5" t="s">
         <v>92</v>
       </c>
-      <c r="E84" s="6" t="s">
+      <c r="E84" s="5" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A85" s="5" t="s">
+    <row r="85" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A85" s="4" t="s">
         <v>81</v>
       </c>
-      <c r="B85" s="6" t="s">
+      <c r="B85" s="5" t="s">
         <v>87</v>
       </c>
-      <c r="C85" s="6" t="s">
+      <c r="C85" s="5" t="s">
         <v>88</v>
       </c>
-      <c r="D85" s="6" t="s">
+      <c r="D85" s="5" t="s">
         <v>89</v>
       </c>
-      <c r="E85" s="6" t="s">
+      <c r="E85" s="5" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A86" s="5"/>
-      <c r="B86" s="6"/>
-      <c r="C86" s="6"/>
-      <c r="D86" s="6"/>
-      <c r="E86" s="6"/>
-    </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A87" s="5" t="s">
+    <row r="86" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A86" s="4"/>
+      <c r="B86" s="5"/>
+      <c r="C86" s="5"/>
+      <c r="D86" s="5"/>
+      <c r="E86" s="5"/>
+    </row>
+    <row r="87" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A87" s="4" t="s">
         <v>105</v>
       </c>
-      <c r="B87" s="6"/>
-      <c r="C87" s="6"/>
-      <c r="D87" s="6"/>
-      <c r="E87" s="6"/>
-    </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A88" s="3" t="s">
+      <c r="B87" s="5"/>
+      <c r="C87" s="5"/>
+      <c r="D87" s="5"/>
+      <c r="E87" s="5"/>
+    </row>
+    <row r="88" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A88" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="B88" s="4" t="s">
+      <c r="B88" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="C88" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="D88" s="4" t="s">
+      <c r="C88" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="D88" s="3" t="s">
         <v>83</v>
       </c>
-      <c r="E88" s="4" t="s">
+      <c r="E88" s="3" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A89" s="5" t="s">
+    <row r="89" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A89" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="B89" s="6" t="s">
+      <c r="B89" s="5" t="s">
         <v>97</v>
       </c>
-      <c r="C89" s="6" t="s">
+      <c r="C89" s="5" t="s">
         <v>88</v>
       </c>
-      <c r="D89" s="6" t="s">
+      <c r="D89" s="5" t="s">
         <v>98</v>
       </c>
-      <c r="E89" s="6" t="s">
+      <c r="E89" s="5" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A91" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="B91" s="6" t="s">
+    <row r="91" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A91" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B91" s="5" t="s">
         <v>100</v>
       </c>
-      <c r="C91" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="D91" s="6" t="s">
+      <c r="C91" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="D91" s="5" t="s">
         <v>92</v>
       </c>
-      <c r="E91" s="6" t="s">
+      <c r="E91" s="5" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A92" s="3" t="s">
+    <row r="92" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A92" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="B92" s="4" t="s">
+      <c r="B92" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="C92" s="4" t="s">
+      <c r="C92" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="D92" s="4" t="s">
+      <c r="D92" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="E92" s="4" t="s">
+      <c r="E92" s="3" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="93" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A93" s="3" t="s">
+    <row r="93" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A93" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="B93" s="4" t="s">
+      <c r="B93" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="C93" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="D93" s="4" t="s">
+      <c r="C93" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="D93" s="3" t="s">
         <v>83</v>
       </c>
-      <c r="E93" s="4" t="s">
+      <c r="E93" s="3" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="94" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A94" s="3" t="s">
+    <row r="94" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A94" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="B94" s="4" t="s">
+      <c r="B94" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="C94" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="D94" s="4" t="s">
+      <c r="C94" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="D94" s="3" t="s">
         <v>83</v>
       </c>
-      <c r="E94" s="4" t="s">
+      <c r="E94" s="3" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="99" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A99" s="3" t="s">
+    <row r="95" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="Q95" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="R95" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="S95" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="T95" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="U95" s="3" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="96" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A96" t="s">
+        <v>108</v>
+      </c>
+      <c r="Q96" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="R96" s="5" t="s">
+        <v>100</v>
+      </c>
+      <c r="S96" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="T96" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="U96" s="5" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="97" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A97" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="B99" s="4" t="s">
+      <c r="B97" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="C99" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="D99" s="4" t="s">
+      <c r="C97" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="D97" s="3" t="s">
         <v>83</v>
       </c>
-      <c r="E99" s="4" t="s">
+      <c r="E97" s="3" t="s">
         <v>106</v>
       </c>
-      <c r="F99" s="7">
+      <c r="F97" s="6">
         <v>44261.745891203704</v>
       </c>
-    </row>
-    <row r="100" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A100" s="3" t="s">
+      <c r="Q97" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="R97" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="S97" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="T97" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="U97" s="3" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="98" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A98" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="B100" s="4" t="s">
+      <c r="B98" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="C100" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="D100" s="4" t="s">
+      <c r="C98" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="D98" s="3" t="s">
         <v>83</v>
       </c>
-      <c r="E100" s="4" t="s">
+      <c r="E98" s="3" t="s">
         <v>107</v>
       </c>
-      <c r="F100" s="7">
+      <c r="F98" s="6">
         <v>44261.746122685188</v>
+      </c>
+      <c r="Q98" s="2"/>
+      <c r="R98" s="3"/>
+      <c r="S98" s="3"/>
+      <c r="T98" s="3"/>
+      <c r="U98" s="3"/>
+    </row>
+    <row r="99" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="Q99" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="R99" s="5" t="s">
+        <v>114</v>
+      </c>
+      <c r="S99" s="5" t="s">
+        <v>116</v>
+      </c>
+      <c r="T99" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="U99" s="5" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="100" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A100" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="101" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A101" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="B101" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="C101" s="3" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="102" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A102" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="B102" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="C102" s="3" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="103" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A103" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="B103" s="5" t="s">
+        <v>121</v>
+      </c>
+      <c r="C103" s="5" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="104" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A104" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="B104" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="C104" s="3" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="105" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A105" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B105" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="C105" s="3" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="106" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A106" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="B106" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="C106" s="5" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="108" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A108" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="109" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A109" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="B109" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="C109" s="5" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="110" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A110" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B110" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="C110" s="3" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="111" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A111" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="B111" s="5" t="s">
+        <v>128</v>
+      </c>
+      <c r="C111" s="5" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="112" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A112" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="B112" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="C112" s="3" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="113" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A113" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B113" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="C113" s="5" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="115" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A115" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="116" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A116" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B116" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="C116" s="3" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="117" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A117" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="B117" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="C117" s="5" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="118" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A118" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="B118" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="C118" s="3" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="120" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A120" t="s">
+        <v>136</v>
+      </c>
+      <c r="Q120" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="R120" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="S120" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="T120" s="6">
+        <v>44266.352488425924</v>
+      </c>
+    </row>
+    <row r="121" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A121" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="B121" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="C121" s="3" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="122" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A122" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="B122" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C122" s="5" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="123" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A123" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="B123" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="C123" s="3" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="124" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A124" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="B124" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C124" s="5" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="126" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A126" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="127" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A127" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B127" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="C127" s="3" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="128" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A128" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="129" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A129" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="B129" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="C129" s="5" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="130" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A130" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="B130" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="C130" s="3" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="131" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A131" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="B131" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="C131" s="5" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="132" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A132" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="B132" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="C132" s="3" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="133" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A133" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="B133" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="C133" s="5" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="134" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A134" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B134" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C134" s="3" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="135" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A135" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="B135" s="5" t="s">
+        <v>113</v>
+      </c>
+      <c r="C135" s="5" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="136" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A136" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="B136" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="C136" s="3" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="138" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A138" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="139" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A139" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="B139" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="C139" s="3" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="140" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A140" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="B140" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C140" s="5" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="141" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A141" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="B141" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="C141" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="143" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A143" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="144" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="N144" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="O144" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="P144" s="3" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="145" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A145" t="s">
+        <v>158</v>
+      </c>
+      <c r="N145" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="O145" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="P145" s="3" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="146" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A146" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="B146" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="C146" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="N146" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="O146" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="P146" s="5" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="147" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A147" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B147" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="C147" s="3" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="148" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A148" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="B148" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="C148" s="5" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="149" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A149" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="B149" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="C149" s="3" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="151" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A151" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="153" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A153" t="s">
+        <v>166</v>
+      </c>
+      <c r="N153" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="O153" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="P153" s="3" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="154" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A154" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="B154" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="C154" s="5" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="155" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A155" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="B155" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="C155" s="5" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="156" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A156" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="B156" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C156" s="5" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="157" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A157" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B157" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="C157" s="5" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="158" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A158" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="B158" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C158" s="3" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="159" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A159" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B159" s="5" t="s">
+        <v>133</v>
+      </c>
+      <c r="C159" s="5" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="160" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A160" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="B160" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C160" s="3" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="161" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A161" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B161" s="5" t="s">
+        <v>133</v>
+      </c>
+      <c r="C161" s="5" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="163" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A163" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="164" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A164" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="B164" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="C164" s="5" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="165" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A165" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B165" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="C165" s="5" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="166" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A166" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B166" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="C166" s="5" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="167" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A167" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="B167" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C167" s="3" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="168" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A168" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="B168" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="C168" s="3" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="170" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A170" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B170" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="C170" s="3" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="172" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A172" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="173" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A173" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="B173" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C173" s="3" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="175" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A175" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="176" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A176" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="B176" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="C176" s="3" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="177" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A177" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="B177" s="5" t="s">
+        <v>113</v>
+      </c>
+      <c r="C177" s="5" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="178" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A178" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B178" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C178" s="5" t="s">
+        <v>187</v>
+      </c>
+      <c r="H178" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="179" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A179" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="B179" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="C179" s="5" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="180" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A180" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B180" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="C180" s="3" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="182" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A182" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="183" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A183" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="B183" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="C183" s="5" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="184" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A184" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="B184" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C184" s="3" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="185" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A185" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B185" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C185" s="5" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="186" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A186" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B186" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="C186" s="3" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="187" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A187" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B187" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="C187" s="5" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="188" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A188" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="B188" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="C188" s="3" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="189" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A189" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="B189" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C189" s="5" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="190" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A190" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B190" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="C190" s="3" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="191" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A191" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="B191" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C191" s="5" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="192" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A192" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B192" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C192" s="3" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="194" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A194" s="7" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="195" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A195" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B195" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C195" s="3" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="197" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A197" s="7" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="198" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A198" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="B198" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="C198" s="3" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="199" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A199" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="B199" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="C199" s="5" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="200" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A200" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="B200" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="C200" s="5" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="201" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A201" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="B201" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="C201" s="3" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="203" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A203" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="204" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A204" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="B204" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="C204" s="5" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="205" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A205" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B205" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="C205" s="5" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="206" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A206" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="B206" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="C206" s="3" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="207" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A207" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B207" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="C207" s="5" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="208" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A208" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="B208" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="C208" s="3" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="209" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A209" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B209" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="C209" s="3" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="210" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A210" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B210" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="C210" s="3" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="212" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A212" s="7" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="213" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A213" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="B213" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="C213" s="5" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="214" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A214" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="B214" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="C214" s="5" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="216" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A216" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="217" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A217" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="B217" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="C217" s="5" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="218" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A218" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="B218" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C218" s="3" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="220" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A220" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="221" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A221" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="B221" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="C221" s="3" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="222" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A222" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B222" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="C222" s="5" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="223" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A223" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="B223" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="C223" s="3" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="224" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A224" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="B224" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C224" s="5" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="225" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A225" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="B225" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="C225" s="3" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="226" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A226" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B226" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="C226" s="3" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="227" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A227" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="B227" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="C227" s="5" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="229" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A229" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="230" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A230" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="B230" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C230" s="3" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="232" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A232" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="233" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A233" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B233" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="C233" s="3" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="234" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A234" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B234" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="C234" s="5" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="235" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A235" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B235" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="C235" s="3" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="236" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A236" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B236" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="C236" s="5" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="237" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A237" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="B237" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C237" s="3" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="238" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A238" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="B238" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="C238" s="5" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="239" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A239" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B239" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C239" s="3" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="240" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A240" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B240" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="C240" s="3" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="241" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A241" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="B241" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="C241" s="5" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="243" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A243" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="244" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A244" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="B244" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C244" s="5" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="245" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A245" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B245" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="C245" s="3" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="247" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A247" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="248" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A248" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="B248" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C248" s="3" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="249" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A249" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="B249" s="3" t="s">
+        <v>242</v>
+      </c>
+      <c r="C249" s="3" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="250" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A250" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="B250" s="5" t="s">
+        <v>150</v>
+      </c>
+      <c r="C250" s="5" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="251" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A251" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="B251" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="C251" s="5" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="252" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A252" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B252" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="C252" s="3" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="254" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A254" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="255" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A255" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="B255" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="C255" s="3" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="256" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A256" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="B256" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="C256" s="5" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="257" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A257" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B257" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="C257" s="3" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="258" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A258" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B258" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="C258" s="5" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="259" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A259" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B259" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="C259" s="3" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="260" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A260" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B260" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="C260" s="5" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="262" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A262" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="B262" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="C262" s="5" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="263" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A263" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="B263" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="C263" s="3" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="264" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A264" s="2" t="s">
+        <v>253</v>
+      </c>
+      <c r="B264" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="C264" s="3" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="266" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A266" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="267" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A267" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B267" s="5" t="s">
+        <v>133</v>
+      </c>
+      <c r="C267" s="5" t="s">
+        <v>256</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Changes to Excel + GeoMaps
</commit_message>
<xml_diff>
--- a/Zeitstrahl.xlsx
+++ b/Zeitstrahl.xlsx
@@ -1,20 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27726"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27830"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\amonb\OneDrive\Dokumente\Semester II\Der Sachverstädnige vor Gericht\Git Repository\sachverst-ndiger\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="A:\HSMW\2. Semester\Sachverständiger\sachverst-ndiger\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D2E797F-078D-4376-A5BC-D5F7FB9CC032}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{328C5A7F-0C6D-4C0F-8AB9-9FF0AEE94DFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{F14C7C15-811B-4F1F-80F2-413CDD7532BB}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{F14C7C15-811B-4F1F-80F2-413CDD7532BB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$45:$A$54</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -888,7 +891,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="22" fontId="0" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1225,6 +1228,13 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{419F6C20-9CB3-4D32-915F-78A5F233F1E4}">
   <dimension ref="A1:U267"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="100" customWidth="1"/>
+    <col min="2" max="2" width="36" customWidth="1"/>
+    <col min="3" max="3" width="21.7109375" customWidth="1"/>
+    <col min="4" max="4" width="32" customWidth="1"/>
+    <col min="5" max="5" width="93.7109375" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">

</xml_diff>